<commit_message>
Add DingTalk webhooks, OAuth hardening, and Excel sheet fidelity fixes.
Real-time webhook endpoints with signature verification, async processing, audit logging, and an admin UI keep attendance in sync automatically; also improves sign/situation sheets and DingTalk login configuration.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/backend/templates/master_template.xlsx
+++ b/backend/templates/master_template.xlsx
@@ -108,17 +108,17 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -490,7 +490,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AX35"/>
+  <dimension ref="A1:AT35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -538,7 +538,6 @@
     <col width="4" customWidth="1" min="43" max="43"/>
     <col width="4" customWidth="1" min="44" max="44"/>
     <col width="4" customWidth="1" min="45" max="45"/>
-    <col width="4" customWidth="1" min="46" max="46"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -548,6 +547,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -564,147 +564,186 @@
           <t>时间</t>
         </is>
       </c>
-      <c r="D3" s="3" t="n"/>
-      <c r="E3" s="3" t="n"/>
-      <c r="F3" s="3" t="n"/>
-      <c r="G3" s="3" t="n"/>
-      <c r="H3" s="3" t="n"/>
-      <c r="I3" s="3" t="n"/>
-      <c r="J3" s="3" t="n"/>
-      <c r="K3" s="3" t="n"/>
-      <c r="L3" s="3" t="n"/>
-      <c r="M3" s="3" t="n"/>
-      <c r="N3" s="3" t="n"/>
-      <c r="O3" s="3" t="n"/>
-      <c r="P3" s="3" t="n"/>
-      <c r="Q3" s="3" t="n"/>
-      <c r="R3" s="3" t="n"/>
-      <c r="S3" s="3" t="n"/>
-      <c r="T3" s="3" t="n"/>
-      <c r="U3" s="3" t="n"/>
-      <c r="V3" s="3" t="n"/>
-      <c r="W3" s="3" t="n"/>
-      <c r="X3" s="3" t="n"/>
-      <c r="Y3" s="3" t="n"/>
-      <c r="Z3" s="3" t="n"/>
-      <c r="AA3" s="3" t="n"/>
-      <c r="AB3" s="3" t="n"/>
-      <c r="AC3" s="3" t="n"/>
-      <c r="AD3" s="3" t="n"/>
-      <c r="AE3" s="3" t="n"/>
-      <c r="AF3" s="3" t="n"/>
-      <c r="AG3" s="3" t="n"/>
-      <c r="AH3" s="3" t="n"/>
+      <c r="D3" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F3" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="G3" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="H3" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="I3" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="J3" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="K3" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="L3" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="M3" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="N3" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="O3" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="P3" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="Q3" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="R3" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="S3" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="T3" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="U3" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="V3" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="W3" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="X3" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="Y3" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="Z3" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="AA3" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="AB3" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="AC3" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="AD3" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="AE3" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="AF3" s="2" t="n">
+        <v>29</v>
+      </c>
+      <c r="AG3" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="AH3" s="2" t="n">
+        <v>31</v>
+      </c>
       <c r="AI3" s="3" t="n"/>
-      <c r="AJ3" s="3" t="n"/>
-      <c r="AK3" s="3" t="n"/>
-      <c r="AL3" s="3" t="n"/>
-      <c r="AM3" s="3" t="n"/>
-      <c r="AN3" s="3" t="n"/>
-      <c r="AO3" s="3" t="n"/>
-      <c r="AP3" s="3" t="n"/>
-      <c r="AQ3" s="3" t="n"/>
-      <c r="AR3" s="3" t="n"/>
-      <c r="AS3" s="3" t="n"/>
-      <c r="AT3" s="3" t="n"/>
+      <c r="AJ3" s="2" t="inlineStr">
+        <is>
+          <t>出勤合计</t>
+        </is>
+      </c>
+      <c r="AK3" s="2" t="inlineStr">
+        <is>
+          <t>事假</t>
+        </is>
+      </c>
+      <c r="AL3" s="2" t="inlineStr">
+        <is>
+          <t>调休</t>
+        </is>
+      </c>
+      <c r="AM3" s="2" t="inlineStr">
+        <is>
+          <t>出差</t>
+        </is>
+      </c>
+      <c r="AN3" s="2" t="inlineStr">
+        <is>
+          <t>病假</t>
+        </is>
+      </c>
+      <c r="AO3" s="2" t="inlineStr">
+        <is>
+          <t>福利假</t>
+        </is>
+      </c>
+      <c r="AP3" s="2" t="inlineStr">
+        <is>
+          <t>年假</t>
+        </is>
+      </c>
+      <c r="AQ3" s="2" t="inlineStr">
+        <is>
+          <t>产假/陪产假</t>
+        </is>
+      </c>
+      <c r="AR3" s="2" t="inlineStr">
+        <is>
+          <t>丧假</t>
+        </is>
+      </c>
+      <c r="AS3" s="2" t="inlineStr">
+        <is>
+          <t>合计</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="n"/>
       <c r="B4" s="3" t="n"/>
       <c r="C4" s="3" t="n"/>
-      <c r="D4" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="E4" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="F4" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="G4" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="H4" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="I4" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="J4" s="2" t="n">
-        <v>7</v>
-      </c>
-      <c r="K4" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="L4" s="2" t="n">
-        <v>9</v>
-      </c>
-      <c r="M4" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="N4" s="2" t="n">
-        <v>11</v>
-      </c>
-      <c r="O4" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="P4" s="2" t="n">
-        <v>13</v>
-      </c>
-      <c r="Q4" s="2" t="n">
-        <v>14</v>
-      </c>
-      <c r="R4" s="2" t="n">
-        <v>15</v>
-      </c>
-      <c r="S4" s="2" t="n">
-        <v>16</v>
-      </c>
-      <c r="T4" s="2" t="n">
-        <v>17</v>
-      </c>
-      <c r="U4" s="2" t="n">
-        <v>18</v>
-      </c>
-      <c r="V4" s="2" t="n">
-        <v>19</v>
-      </c>
-      <c r="W4" s="2" t="n">
-        <v>20</v>
-      </c>
-      <c r="X4" s="2" t="n">
-        <v>21</v>
-      </c>
-      <c r="Y4" s="2" t="n">
-        <v>22</v>
-      </c>
-      <c r="Z4" s="2" t="n">
-        <v>23</v>
-      </c>
-      <c r="AA4" s="2" t="n">
-        <v>24</v>
-      </c>
-      <c r="AB4" s="2" t="n">
-        <v>25</v>
-      </c>
-      <c r="AC4" s="2" t="n">
-        <v>26</v>
-      </c>
-      <c r="AD4" s="2" t="n">
-        <v>27</v>
-      </c>
-      <c r="AE4" s="2" t="n">
-        <v>28</v>
-      </c>
-      <c r="AF4" s="2" t="n">
-        <v>29</v>
-      </c>
-      <c r="AG4" s="2" t="n">
-        <v>30</v>
-      </c>
-      <c r="AH4" s="2" t="n">
-        <v>31</v>
-      </c>
+      <c r="D4" s="3" t="n"/>
+      <c r="E4" s="3" t="n"/>
+      <c r="F4" s="3" t="n"/>
+      <c r="G4" s="3" t="n"/>
+      <c r="H4" s="3" t="n"/>
+      <c r="I4" s="3" t="n"/>
+      <c r="J4" s="3" t="n"/>
+      <c r="K4" s="3" t="n"/>
+      <c r="L4" s="3" t="n"/>
+      <c r="M4" s="3" t="n"/>
+      <c r="N4" s="3" t="n"/>
+      <c r="O4" s="3" t="n"/>
+      <c r="P4" s="3" t="n"/>
+      <c r="Q4" s="3" t="n"/>
+      <c r="R4" s="3" t="n"/>
+      <c r="S4" s="3" t="n"/>
+      <c r="T4" s="3" t="n"/>
+      <c r="U4" s="3" t="n"/>
+      <c r="V4" s="3" t="n"/>
+      <c r="W4" s="3" t="n"/>
+      <c r="X4" s="3" t="n"/>
+      <c r="Y4" s="3" t="n"/>
+      <c r="Z4" s="3" t="n"/>
+      <c r="AA4" s="3" t="n"/>
+      <c r="AB4" s="3" t="n"/>
+      <c r="AC4" s="3" t="n"/>
+      <c r="AD4" s="3" t="n"/>
+      <c r="AE4" s="3" t="n"/>
+      <c r="AF4" s="3" t="n"/>
+      <c r="AG4" s="3" t="n"/>
+      <c r="AH4" s="3" t="n"/>
       <c r="AI4" s="3" t="n"/>
       <c r="AJ4" s="3" t="n"/>
       <c r="AK4" s="3" t="n"/>
@@ -716,11 +755,6 @@
       <c r="AQ4" s="3" t="n"/>
       <c r="AR4" s="3" t="n"/>
       <c r="AS4" s="3" t="n"/>
-      <c r="AT4" s="2" t="inlineStr">
-        <is>
-          <t>缺勤</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="n"/>
@@ -808,7 +842,6 @@
           <t>ML (婚假)</t>
         </is>
       </c>
-      <c r="AT5" s="3" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n"/>
@@ -886,8 +919,7 @@
         <f>COUNTIF(D6:AH6,$AR$5)</f>
         <v/>
       </c>
-      <c r="AS6" s="3" t="n"/>
-      <c r="AT6" s="4">
+      <c r="AS6" s="4">
         <f>21-AJ6</f>
         <v/>
       </c>
@@ -968,8 +1000,7 @@
         <f>COUNTIF(D7:AH7,$AR$5)</f>
         <v/>
       </c>
-      <c r="AS7" s="3" t="n"/>
-      <c r="AT7" s="4">
+      <c r="AS7" s="4">
         <f>21-AJ7</f>
         <v/>
       </c>
@@ -1050,8 +1081,7 @@
         <f>COUNTIF(D8:AH8,$AR$5)</f>
         <v/>
       </c>
-      <c r="AS8" s="3" t="n"/>
-      <c r="AT8" s="4">
+      <c r="AS8" s="4">
         <f>21-AJ8</f>
         <v/>
       </c>
@@ -1132,8 +1162,7 @@
         <f>COUNTIF(D9:AH9,$AR$5)</f>
         <v/>
       </c>
-      <c r="AS9" s="3" t="n"/>
-      <c r="AT9" s="4">
+      <c r="AS9" s="4">
         <f>21-AJ9</f>
         <v/>
       </c>
@@ -1214,8 +1243,7 @@
         <f>COUNTIF(D10:AH10,$AR$5)</f>
         <v/>
       </c>
-      <c r="AS10" s="3" t="n"/>
-      <c r="AT10" s="4">
+      <c r="AS10" s="4">
         <f>21-AJ10</f>
         <v/>
       </c>
@@ -1296,8 +1324,7 @@
         <f>COUNTIF(D11:AH11,$AR$5)</f>
         <v/>
       </c>
-      <c r="AS11" s="3" t="n"/>
-      <c r="AT11" s="4">
+      <c r="AS11" s="4">
         <f>21-AJ11</f>
         <v/>
       </c>
@@ -1378,8 +1405,7 @@
         <f>COUNTIF(D12:AH12,$AR$5)</f>
         <v/>
       </c>
-      <c r="AS12" s="3" t="n"/>
-      <c r="AT12" s="4">
+      <c r="AS12" s="4">
         <f>21-AJ12</f>
         <v/>
       </c>
@@ -1460,8 +1486,7 @@
         <f>COUNTIF(D13:AH13,$AR$5)</f>
         <v/>
       </c>
-      <c r="AS13" s="3" t="n"/>
-      <c r="AT13" s="4">
+      <c r="AS13" s="4">
         <f>21-AJ13</f>
         <v/>
       </c>
@@ -1542,8 +1567,7 @@
         <f>COUNTIF(D14:AH14,$AR$5)</f>
         <v/>
       </c>
-      <c r="AS14" s="3" t="n"/>
-      <c r="AT14" s="4">
+      <c r="AS14" s="4">
         <f>21-AJ14</f>
         <v/>
       </c>
@@ -1624,8 +1648,7 @@
         <f>COUNTIF(D15:AH15,$AR$5)</f>
         <v/>
       </c>
-      <c r="AS15" s="3" t="n"/>
-      <c r="AT15" s="4">
+      <c r="AS15" s="4">
         <f>21-AJ15</f>
         <v/>
       </c>
@@ -1706,8 +1729,7 @@
         <f>COUNTIF(D16:AH16,$AR$5)</f>
         <v/>
       </c>
-      <c r="AS16" s="3" t="n"/>
-      <c r="AT16" s="4">
+      <c r="AS16" s="4">
         <f>21-AJ16</f>
         <v/>
       </c>
@@ -1788,8 +1810,7 @@
         <f>COUNTIF(D17:AH17,$AR$5)</f>
         <v/>
       </c>
-      <c r="AS17" s="3" t="n"/>
-      <c r="AT17" s="4">
+      <c r="AS17" s="4">
         <f>21-AJ17</f>
         <v/>
       </c>
@@ -1870,8 +1891,7 @@
         <f>COUNTIF(D18:AH18,$AR$5)</f>
         <v/>
       </c>
-      <c r="AS18" s="3" t="n"/>
-      <c r="AT18" s="4">
+      <c r="AS18" s="4">
         <f>21-AJ18</f>
         <v/>
       </c>
@@ -1952,8 +1972,7 @@
         <f>COUNTIF(D19:AH19,$AR$5)</f>
         <v/>
       </c>
-      <c r="AS19" s="3" t="n"/>
-      <c r="AT19" s="4">
+      <c r="AS19" s="4">
         <f>21-AJ19</f>
         <v/>
       </c>
@@ -2034,8 +2053,7 @@
         <f>COUNTIF(D20:AH20,$AR$5)</f>
         <v/>
       </c>
-      <c r="AS20" s="3" t="n"/>
-      <c r="AT20" s="4">
+      <c r="AS20" s="4">
         <f>21-AJ20</f>
         <v/>
       </c>
@@ -2116,8 +2134,7 @@
         <f>COUNTIF(D21:AH21,$AR$5)</f>
         <v/>
       </c>
-      <c r="AS21" s="3" t="n"/>
-      <c r="AT21" s="4">
+      <c r="AS21" s="4">
         <f>21-AJ21</f>
         <v/>
       </c>
@@ -2198,8 +2215,7 @@
         <f>COUNTIF(D22:AH22,$AR$5)</f>
         <v/>
       </c>
-      <c r="AS22" s="3" t="n"/>
-      <c r="AT22" s="4">
+      <c r="AS22" s="4">
         <f>21-AJ22</f>
         <v/>
       </c>
@@ -2280,8 +2296,7 @@
         <f>COUNTIF(D23:AH23,$AR$5)</f>
         <v/>
       </c>
-      <c r="AS23" s="3" t="n"/>
-      <c r="AT23" s="4">
+      <c r="AS23" s="4">
         <f>21-AJ23</f>
         <v/>
       </c>
@@ -2362,8 +2377,7 @@
         <f>COUNTIF(D24:AH24,$AR$5)</f>
         <v/>
       </c>
-      <c r="AS24" s="3" t="n"/>
-      <c r="AT24" s="4">
+      <c r="AS24" s="4">
         <f>21-AJ24</f>
         <v/>
       </c>
@@ -2444,8 +2458,7 @@
         <f>COUNTIF(D25:AH25,$AR$5)</f>
         <v/>
       </c>
-      <c r="AS25" s="3" t="n"/>
-      <c r="AT25" s="4">
+      <c r="AS25" s="4">
         <f>21-AJ25</f>
         <v/>
       </c>
@@ -2526,8 +2539,7 @@
         <f>COUNTIF(D26:AH26,$AR$5)</f>
         <v/>
       </c>
-      <c r="AS26" s="3" t="n"/>
-      <c r="AT26" s="4">
+      <c r="AS26" s="4">
         <f>21-AJ26</f>
         <v/>
       </c>
@@ -2608,8 +2620,7 @@
         <f>COUNTIF(D27:AH27,$AR$5)</f>
         <v/>
       </c>
-      <c r="AS27" s="3" t="n"/>
-      <c r="AT27" s="4">
+      <c r="AS27" s="4">
         <f>21-AJ27</f>
         <v/>
       </c>
@@ -2690,8 +2701,7 @@
         <f>COUNTIF(D28:AH28,$AR$5)</f>
         <v/>
       </c>
-      <c r="AS28" s="3" t="n"/>
-      <c r="AT28" s="4">
+      <c r="AS28" s="4">
         <f>21-AJ28</f>
         <v/>
       </c>
@@ -2772,8 +2782,7 @@
         <f>COUNTIF(D29:AH29,$AR$5)</f>
         <v/>
       </c>
-      <c r="AS29" s="3" t="n"/>
-      <c r="AT29" s="4">
+      <c r="AS29" s="4">
         <f>21-AJ29</f>
         <v/>
       </c>
@@ -2854,8 +2863,7 @@
         <f>COUNTIF(D30:AH30,$AR$5)</f>
         <v/>
       </c>
-      <c r="AS30" s="3" t="n"/>
-      <c r="AT30" s="4">
+      <c r="AS30" s="4">
         <f>21-AJ30</f>
         <v/>
       </c>
@@ -2936,8 +2944,7 @@
         <f>COUNTIF(D31:AH31,$AR$5)</f>
         <v/>
       </c>
-      <c r="AS31" s="3" t="n"/>
-      <c r="AT31" s="4">
+      <c r="AS31" s="4">
         <f>21-AJ31</f>
         <v/>
       </c>
@@ -3018,8 +3025,7 @@
         <f>COUNTIF(D32:AH32,$AR$5)</f>
         <v/>
       </c>
-      <c r="AS32" s="3" t="n"/>
-      <c r="AT32" s="4">
+      <c r="AS32" s="4">
         <f>21-AJ32</f>
         <v/>
       </c>
@@ -3100,8 +3106,7 @@
         <f>COUNTIF(D33:AH33,$AR$5)</f>
         <v/>
       </c>
-      <c r="AS33" s="3" t="n"/>
-      <c r="AT33" s="4">
+      <c r="AS33" s="4">
         <f>21-AJ33</f>
         <v/>
       </c>
@@ -3182,8 +3187,7 @@
         <f>COUNTIF(D34:AH34,$AR$5)</f>
         <v/>
       </c>
-      <c r="AS34" s="3" t="n"/>
-      <c r="AT34" s="4">
+      <c r="AS34" s="4">
         <f>21-AJ34</f>
         <v/>
       </c>
@@ -3264,8 +3268,7 @@
         <f>COUNTIF(D35:AH35,$AR$5)</f>
         <v/>
       </c>
-      <c r="AS35" s="3" t="n"/>
-      <c r="AT35" s="4">
+      <c r="AS35" s="4">
         <f>21-AJ35</f>
         <v/>
       </c>
@@ -3281,7 +3284,6 @@
     <mergeCell ref="B14:B15"/>
     <mergeCell ref="A12:A13"/>
     <mergeCell ref="A26:A27"/>
-    <mergeCell ref="A1:AX1"/>
     <mergeCell ref="B34:B35"/>
     <mergeCell ref="B10:B11"/>
     <mergeCell ref="B28:B29"/>
@@ -3295,6 +3297,7 @@
     <mergeCell ref="A20:A21"/>
     <mergeCell ref="B20:B21"/>
     <mergeCell ref="A10:A11"/>
+    <mergeCell ref="A1:AT1"/>
     <mergeCell ref="B30:B31"/>
     <mergeCell ref="B32:B33"/>
     <mergeCell ref="A34:A35"/>
@@ -3712,7 +3715,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF19"/>
+  <dimension ref="A1:AF18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -3755,918 +3758,751 @@
           <t>月度汇总 统计日期：2026-05-01 至 2026-05-31</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="C1" s="7" t="inlineStr">
-        <is>
-          <t>六</t>
-        </is>
-      </c>
-      <c r="D1" s="7" t="inlineStr">
-        <is>
-          <t>日</t>
-        </is>
-      </c>
-      <c r="E1" s="2" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="F1" s="2" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="G1" s="2" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="H1" s="2" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="I1" s="2" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="J1" s="7" t="inlineStr">
-        <is>
-          <t>六</t>
-        </is>
-      </c>
-      <c r="K1" s="7" t="inlineStr">
-        <is>
-          <t>日</t>
-        </is>
-      </c>
-      <c r="L1" s="2" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="M1" s="2" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
-      </c>
-      <c r="N1" s="2" t="inlineStr">
-        <is>
-          <t>13</t>
-        </is>
-      </c>
-      <c r="O1" s="2" t="inlineStr">
-        <is>
-          <t>14</t>
-        </is>
-      </c>
-      <c r="P1" s="2" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
-      </c>
-      <c r="Q1" s="7" t="inlineStr">
-        <is>
-          <t>六</t>
-        </is>
-      </c>
-      <c r="R1" s="7" t="inlineStr">
-        <is>
-          <t>日</t>
-        </is>
-      </c>
-      <c r="S1" s="2" t="inlineStr">
-        <is>
-          <t>18</t>
-        </is>
-      </c>
-      <c r="T1" s="2" t="inlineStr">
-        <is>
-          <t>19</t>
-        </is>
-      </c>
-      <c r="U1" s="2" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
-      <c r="V1" s="2" t="inlineStr">
-        <is>
-          <t>21</t>
-        </is>
-      </c>
-      <c r="W1" s="2" t="inlineStr">
-        <is>
-          <t>22</t>
-        </is>
-      </c>
-      <c r="X1" s="7" t="inlineStr">
-        <is>
-          <t>六</t>
-        </is>
-      </c>
-      <c r="Y1" s="7" t="inlineStr">
-        <is>
-          <t>日</t>
-        </is>
-      </c>
-      <c r="Z1" s="2" t="inlineStr">
-        <is>
-          <t>25</t>
-        </is>
-      </c>
-      <c r="AA1" s="2" t="inlineStr">
-        <is>
-          <t>26</t>
-        </is>
-      </c>
-      <c r="AB1" s="2" t="inlineStr">
-        <is>
-          <t>27</t>
-        </is>
-      </c>
-      <c r="AC1" s="2" t="inlineStr">
-        <is>
-          <t>28</t>
-        </is>
-      </c>
-      <c r="AD1" s="2" t="inlineStr">
-        <is>
-          <t>29</t>
-        </is>
-      </c>
-      <c r="AE1" s="7" t="inlineStr">
-        <is>
-          <t>六</t>
-        </is>
-      </c>
-      <c r="AF1" s="7" t="inlineStr">
-        <is>
-          <t>日</t>
-        </is>
-      </c>
+      <c r="B1" s="4" t="n"/>
+      <c r="C1" s="7" t="n"/>
+      <c r="D1" s="7" t="n"/>
+      <c r="E1" s="4" t="n"/>
+      <c r="F1" s="4" t="n"/>
+      <c r="G1" s="4" t="n"/>
+      <c r="H1" s="4" t="n"/>
+      <c r="I1" s="4" t="n"/>
+      <c r="J1" s="7" t="n"/>
+      <c r="K1" s="7" t="n"/>
+      <c r="L1" s="4" t="n"/>
+      <c r="M1" s="4" t="n"/>
+      <c r="N1" s="4" t="n"/>
+      <c r="O1" s="4" t="n"/>
+      <c r="P1" s="4" t="n"/>
+      <c r="Q1" s="7" t="n"/>
+      <c r="R1" s="7" t="n"/>
+      <c r="S1" s="4" t="n"/>
+      <c r="T1" s="4" t="n"/>
+      <c r="U1" s="4" t="n"/>
+      <c r="V1" s="4" t="n"/>
+      <c r="W1" s="4" t="n"/>
+      <c r="X1" s="7" t="n"/>
+      <c r="Y1" s="7" t="n"/>
+      <c r="Z1" s="4" t="n"/>
+      <c r="AA1" s="4" t="n"/>
+      <c r="AB1" s="4" t="n"/>
+      <c r="AC1" s="4" t="n"/>
+      <c r="AD1" s="4" t="n"/>
+      <c r="AE1" s="7" t="n"/>
+      <c r="AF1" s="7" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>报表生成时间：2026-06-17 03:25</t>
+          <t>报表生成时间：2026-06-17 03:50</t>
         </is>
       </c>
       <c r="B2" s="4" t="n"/>
-      <c r="C2" s="9" t="n"/>
-      <c r="D2" s="9" t="n"/>
+      <c r="C2" s="7" t="n"/>
+      <c r="D2" s="7" t="n"/>
       <c r="E2" s="4" t="n"/>
       <c r="F2" s="4" t="n"/>
       <c r="G2" s="4" t="n"/>
       <c r="H2" s="4" t="n"/>
       <c r="I2" s="4" t="n"/>
-      <c r="J2" s="9" t="n"/>
-      <c r="K2" s="9" t="n"/>
+      <c r="J2" s="7" t="n"/>
+      <c r="K2" s="7" t="n"/>
       <c r="L2" s="4" t="n"/>
       <c r="M2" s="4" t="n"/>
       <c r="N2" s="4" t="n"/>
       <c r="O2" s="4" t="n"/>
       <c r="P2" s="4" t="n"/>
-      <c r="Q2" s="9" t="n"/>
-      <c r="R2" s="9" t="n"/>
+      <c r="Q2" s="7" t="n"/>
+      <c r="R2" s="7" t="n"/>
       <c r="S2" s="4" t="n"/>
       <c r="T2" s="4" t="n"/>
       <c r="U2" s="4" t="n"/>
       <c r="V2" s="4" t="n"/>
       <c r="W2" s="4" t="n"/>
-      <c r="X2" s="9" t="n"/>
-      <c r="Y2" s="9" t="n"/>
+      <c r="X2" s="7" t="n"/>
+      <c r="Y2" s="7" t="n"/>
       <c r="Z2" s="4" t="n"/>
       <c r="AA2" s="4" t="n"/>
       <c r="AB2" s="4" t="n"/>
       <c r="AC2" s="4" t="n"/>
       <c r="AD2" s="4" t="n"/>
-      <c r="AE2" s="9" t="n"/>
-      <c r="AF2" s="9" t="n"/>
+      <c r="AE2" s="7" t="n"/>
+      <c r="AF2" s="7" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" s="9" t="inlineStr">
         <is>
           <t>姓名</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>每日考勤状态</t>
-        </is>
-      </c>
-      <c r="C3" s="9" t="n"/>
-      <c r="D3" s="9" t="n"/>
-      <c r="E3" s="4" t="n"/>
-      <c r="F3" s="4" t="n"/>
-      <c r="G3" s="4" t="n"/>
-      <c r="H3" s="4" t="n"/>
-      <c r="I3" s="4" t="n"/>
-      <c r="J3" s="9" t="n"/>
-      <c r="K3" s="9" t="n"/>
-      <c r="L3" s="4" t="n"/>
-      <c r="M3" s="4" t="n"/>
-      <c r="N3" s="4" t="n"/>
-      <c r="O3" s="4" t="n"/>
-      <c r="P3" s="4" t="n"/>
-      <c r="Q3" s="9" t="n"/>
-      <c r="R3" s="9" t="n"/>
-      <c r="S3" s="4" t="n"/>
-      <c r="T3" s="4" t="n"/>
-      <c r="U3" s="4" t="n"/>
-      <c r="V3" s="4" t="n"/>
-      <c r="W3" s="4" t="n"/>
-      <c r="X3" s="9" t="n"/>
-      <c r="Y3" s="9" t="n"/>
-      <c r="Z3" s="4" t="n"/>
-      <c r="AA3" s="4" t="n"/>
-      <c r="AB3" s="4" t="n"/>
-      <c r="AC3" s="4" t="n"/>
-      <c r="AD3" s="4" t="n"/>
-      <c r="AE3" s="9" t="n"/>
-      <c r="AF3" s="9" t="n"/>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C3" s="10" t="inlineStr">
+        <is>
+          <t>六</t>
+        </is>
+      </c>
+      <c r="D3" s="10" t="inlineStr">
+        <is>
+          <t>日</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="J3" s="10" t="inlineStr">
+        <is>
+          <t>六</t>
+        </is>
+      </c>
+      <c r="K3" s="10" t="inlineStr">
+        <is>
+          <t>日</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="O3" s="2" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="P3" s="2" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="Q3" s="10" t="inlineStr">
+        <is>
+          <t>六</t>
+        </is>
+      </c>
+      <c r="R3" s="10" t="inlineStr">
+        <is>
+          <t>日</t>
+        </is>
+      </c>
+      <c r="S3" s="2" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="T3" s="2" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="U3" s="2" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="V3" s="2" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="W3" s="2" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="X3" s="10" t="inlineStr">
+        <is>
+          <t>六</t>
+        </is>
+      </c>
+      <c r="Y3" s="10" t="inlineStr">
+        <is>
+          <t>日</t>
+        </is>
+      </c>
+      <c r="Z3" s="2" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="AA3" s="2" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="AB3" s="2" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="AC3" s="2" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="AD3" s="2" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
+      <c r="AE3" s="10" t="inlineStr">
+        <is>
+          <t>六</t>
+        </is>
+      </c>
+      <c r="AF3" s="10" t="inlineStr">
+        <is>
+          <t>日</t>
+        </is>
+      </c>
     </row>
     <row r="4">
-      <c r="A4" s="10" t="inlineStr">
-        <is>
-          <t>姓名</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="C4" s="7" t="inlineStr">
-        <is>
-          <t>六</t>
-        </is>
-      </c>
-      <c r="D4" s="7" t="inlineStr">
-        <is>
-          <t>日</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="I4" s="2" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="J4" s="7" t="inlineStr">
-        <is>
-          <t>六</t>
-        </is>
-      </c>
-      <c r="K4" s="7" t="inlineStr">
-        <is>
-          <t>日</t>
-        </is>
-      </c>
-      <c r="L4" s="2" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="M4" s="2" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
-      </c>
-      <c r="N4" s="2" t="inlineStr">
-        <is>
-          <t>13</t>
-        </is>
-      </c>
-      <c r="O4" s="2" t="inlineStr">
-        <is>
-          <t>14</t>
-        </is>
-      </c>
-      <c r="P4" s="2" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
-      </c>
-      <c r="Q4" s="7" t="inlineStr">
-        <is>
-          <t>六</t>
-        </is>
-      </c>
-      <c r="R4" s="7" t="inlineStr">
-        <is>
-          <t>日</t>
-        </is>
-      </c>
-      <c r="S4" s="2" t="inlineStr">
-        <is>
-          <t>18</t>
-        </is>
-      </c>
-      <c r="T4" s="2" t="inlineStr">
-        <is>
-          <t>19</t>
-        </is>
-      </c>
-      <c r="U4" s="2" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
-      <c r="V4" s="2" t="inlineStr">
-        <is>
-          <t>21</t>
-        </is>
-      </c>
-      <c r="W4" s="2" t="inlineStr">
-        <is>
-          <t>22</t>
-        </is>
-      </c>
-      <c r="X4" s="7" t="inlineStr">
-        <is>
-          <t>六</t>
-        </is>
-      </c>
-      <c r="Y4" s="7" t="inlineStr">
-        <is>
-          <t>日</t>
-        </is>
-      </c>
-      <c r="Z4" s="2" t="inlineStr">
-        <is>
-          <t>25</t>
-        </is>
-      </c>
-      <c r="AA4" s="2" t="inlineStr">
-        <is>
-          <t>26</t>
-        </is>
-      </c>
-      <c r="AB4" s="2" t="inlineStr">
-        <is>
-          <t>27</t>
-        </is>
-      </c>
-      <c r="AC4" s="2" t="inlineStr">
-        <is>
-          <t>28</t>
-        </is>
-      </c>
-      <c r="AD4" s="2" t="inlineStr">
-        <is>
-          <t>29</t>
-        </is>
-      </c>
-      <c r="AE4" s="7" t="inlineStr">
-        <is>
-          <t>六</t>
-        </is>
-      </c>
-      <c r="AF4" s="7" t="inlineStr">
-        <is>
-          <t>日</t>
-        </is>
-      </c>
+      <c r="A4" s="8" t="n"/>
+      <c r="B4" s="4" t="inlineStr"/>
+      <c r="C4" s="7" t="inlineStr"/>
+      <c r="D4" s="7" t="inlineStr"/>
+      <c r="E4" s="4" t="inlineStr"/>
+      <c r="F4" s="4" t="inlineStr"/>
+      <c r="G4" s="4" t="inlineStr"/>
+      <c r="H4" s="4" t="inlineStr"/>
+      <c r="I4" s="4" t="inlineStr"/>
+      <c r="J4" s="7" t="inlineStr"/>
+      <c r="K4" s="7" t="inlineStr"/>
+      <c r="L4" s="4" t="inlineStr"/>
+      <c r="M4" s="4" t="inlineStr"/>
+      <c r="N4" s="4" t="inlineStr"/>
+      <c r="O4" s="4" t="inlineStr"/>
+      <c r="P4" s="4" t="inlineStr"/>
+      <c r="Q4" s="7" t="inlineStr"/>
+      <c r="R4" s="7" t="inlineStr"/>
+      <c r="S4" s="4" t="inlineStr"/>
+      <c r="T4" s="4" t="inlineStr"/>
+      <c r="U4" s="4" t="inlineStr"/>
+      <c r="V4" s="4" t="inlineStr"/>
+      <c r="W4" s="4" t="inlineStr"/>
+      <c r="X4" s="7" t="inlineStr"/>
+      <c r="Y4" s="7" t="inlineStr"/>
+      <c r="Z4" s="4" t="inlineStr"/>
+      <c r="AA4" s="4" t="inlineStr"/>
+      <c r="AB4" s="4" t="inlineStr"/>
+      <c r="AC4" s="4" t="inlineStr"/>
+      <c r="AD4" s="4" t="inlineStr"/>
+      <c r="AE4" s="7" t="inlineStr"/>
+      <c r="AF4" s="7" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="8" t="n"/>
       <c r="B5" s="4" t="inlineStr"/>
-      <c r="C5" s="9" t="inlineStr"/>
-      <c r="D5" s="9" t="inlineStr"/>
+      <c r="C5" s="7" t="inlineStr"/>
+      <c r="D5" s="7" t="inlineStr"/>
       <c r="E5" s="4" t="inlineStr"/>
       <c r="F5" s="4" t="inlineStr"/>
       <c r="G5" s="4" t="inlineStr"/>
       <c r="H5" s="4" t="inlineStr"/>
       <c r="I5" s="4" t="inlineStr"/>
-      <c r="J5" s="9" t="inlineStr"/>
-      <c r="K5" s="9" t="inlineStr"/>
+      <c r="J5" s="7" t="inlineStr"/>
+      <c r="K5" s="7" t="inlineStr"/>
       <c r="L5" s="4" t="inlineStr"/>
       <c r="M5" s="4" t="inlineStr"/>
       <c r="N5" s="4" t="inlineStr"/>
       <c r="O5" s="4" t="inlineStr"/>
       <c r="P5" s="4" t="inlineStr"/>
-      <c r="Q5" s="9" t="inlineStr"/>
-      <c r="R5" s="9" t="inlineStr"/>
+      <c r="Q5" s="7" t="inlineStr"/>
+      <c r="R5" s="7" t="inlineStr"/>
       <c r="S5" s="4" t="inlineStr"/>
       <c r="T5" s="4" t="inlineStr"/>
       <c r="U5" s="4" t="inlineStr"/>
       <c r="V5" s="4" t="inlineStr"/>
       <c r="W5" s="4" t="inlineStr"/>
-      <c r="X5" s="9" t="inlineStr"/>
-      <c r="Y5" s="9" t="inlineStr"/>
+      <c r="X5" s="7" t="inlineStr"/>
+      <c r="Y5" s="7" t="inlineStr"/>
       <c r="Z5" s="4" t="inlineStr"/>
       <c r="AA5" s="4" t="inlineStr"/>
       <c r="AB5" s="4" t="inlineStr"/>
       <c r="AC5" s="4" t="inlineStr"/>
       <c r="AD5" s="4" t="inlineStr"/>
-      <c r="AE5" s="9" t="inlineStr"/>
-      <c r="AF5" s="9" t="inlineStr"/>
+      <c r="AE5" s="7" t="inlineStr"/>
+      <c r="AF5" s="7" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="8" t="n"/>
       <c r="B6" s="4" t="inlineStr"/>
-      <c r="C6" s="9" t="inlineStr"/>
-      <c r="D6" s="9" t="inlineStr"/>
+      <c r="C6" s="7" t="inlineStr"/>
+      <c r="D6" s="7" t="inlineStr"/>
       <c r="E6" s="4" t="inlineStr"/>
       <c r="F6" s="4" t="inlineStr"/>
       <c r="G6" s="4" t="inlineStr"/>
       <c r="H6" s="4" t="inlineStr"/>
       <c r="I6" s="4" t="inlineStr"/>
-      <c r="J6" s="9" t="inlineStr"/>
-      <c r="K6" s="9" t="inlineStr"/>
+      <c r="J6" s="7" t="inlineStr"/>
+      <c r="K6" s="7" t="inlineStr"/>
       <c r="L6" s="4" t="inlineStr"/>
       <c r="M6" s="4" t="inlineStr"/>
       <c r="N6" s="4" t="inlineStr"/>
       <c r="O6" s="4" t="inlineStr"/>
       <c r="P6" s="4" t="inlineStr"/>
-      <c r="Q6" s="9" t="inlineStr"/>
-      <c r="R6" s="9" t="inlineStr"/>
+      <c r="Q6" s="7" t="inlineStr"/>
+      <c r="R6" s="7" t="inlineStr"/>
       <c r="S6" s="4" t="inlineStr"/>
       <c r="T6" s="4" t="inlineStr"/>
       <c r="U6" s="4" t="inlineStr"/>
       <c r="V6" s="4" t="inlineStr"/>
       <c r="W6" s="4" t="inlineStr"/>
-      <c r="X6" s="9" t="inlineStr"/>
-      <c r="Y6" s="9" t="inlineStr"/>
+      <c r="X6" s="7" t="inlineStr"/>
+      <c r="Y6" s="7" t="inlineStr"/>
       <c r="Z6" s="4" t="inlineStr"/>
       <c r="AA6" s="4" t="inlineStr"/>
       <c r="AB6" s="4" t="inlineStr"/>
       <c r="AC6" s="4" t="inlineStr"/>
       <c r="AD6" s="4" t="inlineStr"/>
-      <c r="AE6" s="9" t="inlineStr"/>
-      <c r="AF6" s="9" t="inlineStr"/>
+      <c r="AE6" s="7" t="inlineStr"/>
+      <c r="AF6" s="7" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="8" t="n"/>
       <c r="B7" s="4" t="inlineStr"/>
-      <c r="C7" s="9" t="inlineStr"/>
-      <c r="D7" s="9" t="inlineStr"/>
+      <c r="C7" s="7" t="inlineStr"/>
+      <c r="D7" s="7" t="inlineStr"/>
       <c r="E7" s="4" t="inlineStr"/>
       <c r="F7" s="4" t="inlineStr"/>
       <c r="G7" s="4" t="inlineStr"/>
       <c r="H7" s="4" t="inlineStr"/>
       <c r="I7" s="4" t="inlineStr"/>
-      <c r="J7" s="9" t="inlineStr"/>
-      <c r="K7" s="9" t="inlineStr"/>
+      <c r="J7" s="7" t="inlineStr"/>
+      <c r="K7" s="7" t="inlineStr"/>
       <c r="L7" s="4" t="inlineStr"/>
       <c r="M7" s="4" t="inlineStr"/>
       <c r="N7" s="4" t="inlineStr"/>
       <c r="O7" s="4" t="inlineStr"/>
       <c r="P7" s="4" t="inlineStr"/>
-      <c r="Q7" s="9" t="inlineStr"/>
-      <c r="R7" s="9" t="inlineStr"/>
+      <c r="Q7" s="7" t="inlineStr"/>
+      <c r="R7" s="7" t="inlineStr"/>
       <c r="S7" s="4" t="inlineStr"/>
       <c r="T7" s="4" t="inlineStr"/>
       <c r="U7" s="4" t="inlineStr"/>
       <c r="V7" s="4" t="inlineStr"/>
       <c r="W7" s="4" t="inlineStr"/>
-      <c r="X7" s="9" t="inlineStr"/>
-      <c r="Y7" s="9" t="inlineStr"/>
+      <c r="X7" s="7" t="inlineStr"/>
+      <c r="Y7" s="7" t="inlineStr"/>
       <c r="Z7" s="4" t="inlineStr"/>
       <c r="AA7" s="4" t="inlineStr"/>
       <c r="AB7" s="4" t="inlineStr"/>
       <c r="AC7" s="4" t="inlineStr"/>
       <c r="AD7" s="4" t="inlineStr"/>
-      <c r="AE7" s="9" t="inlineStr"/>
-      <c r="AF7" s="9" t="inlineStr"/>
+      <c r="AE7" s="7" t="inlineStr"/>
+      <c r="AF7" s="7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="8" t="n"/>
       <c r="B8" s="4" t="inlineStr"/>
-      <c r="C8" s="9" t="inlineStr"/>
-      <c r="D8" s="9" t="inlineStr"/>
+      <c r="C8" s="7" t="inlineStr"/>
+      <c r="D8" s="7" t="inlineStr"/>
       <c r="E8" s="4" t="inlineStr"/>
       <c r="F8" s="4" t="inlineStr"/>
       <c r="G8" s="4" t="inlineStr"/>
       <c r="H8" s="4" t="inlineStr"/>
       <c r="I8" s="4" t="inlineStr"/>
-      <c r="J8" s="9" t="inlineStr"/>
-      <c r="K8" s="9" t="inlineStr"/>
+      <c r="J8" s="7" t="inlineStr"/>
+      <c r="K8" s="7" t="inlineStr"/>
       <c r="L8" s="4" t="inlineStr"/>
       <c r="M8" s="4" t="inlineStr"/>
       <c r="N8" s="4" t="inlineStr"/>
       <c r="O8" s="4" t="inlineStr"/>
       <c r="P8" s="4" t="inlineStr"/>
-      <c r="Q8" s="9" t="inlineStr"/>
-      <c r="R8" s="9" t="inlineStr"/>
+      <c r="Q8" s="7" t="inlineStr"/>
+      <c r="R8" s="7" t="inlineStr"/>
       <c r="S8" s="4" t="inlineStr"/>
       <c r="T8" s="4" t="inlineStr"/>
       <c r="U8" s="4" t="inlineStr"/>
       <c r="V8" s="4" t="inlineStr"/>
       <c r="W8" s="4" t="inlineStr"/>
-      <c r="X8" s="9" t="inlineStr"/>
-      <c r="Y8" s="9" t="inlineStr"/>
+      <c r="X8" s="7" t="inlineStr"/>
+      <c r="Y8" s="7" t="inlineStr"/>
       <c r="Z8" s="4" t="inlineStr"/>
       <c r="AA8" s="4" t="inlineStr"/>
       <c r="AB8" s="4" t="inlineStr"/>
       <c r="AC8" s="4" t="inlineStr"/>
       <c r="AD8" s="4" t="inlineStr"/>
-      <c r="AE8" s="9" t="inlineStr"/>
-      <c r="AF8" s="9" t="inlineStr"/>
+      <c r="AE8" s="7" t="inlineStr"/>
+      <c r="AF8" s="7" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="8" t="n"/>
       <c r="B9" s="4" t="inlineStr"/>
-      <c r="C9" s="9" t="inlineStr"/>
-      <c r="D9" s="9" t="inlineStr"/>
+      <c r="C9" s="7" t="inlineStr"/>
+      <c r="D9" s="7" t="inlineStr"/>
       <c r="E9" s="4" t="inlineStr"/>
       <c r="F9" s="4" t="inlineStr"/>
       <c r="G9" s="4" t="inlineStr"/>
       <c r="H9" s="4" t="inlineStr"/>
       <c r="I9" s="4" t="inlineStr"/>
-      <c r="J9" s="9" t="inlineStr"/>
-      <c r="K9" s="9" t="inlineStr"/>
+      <c r="J9" s="7" t="inlineStr"/>
+      <c r="K9" s="7" t="inlineStr"/>
       <c r="L9" s="4" t="inlineStr"/>
       <c r="M9" s="4" t="inlineStr"/>
       <c r="N9" s="4" t="inlineStr"/>
       <c r="O9" s="4" t="inlineStr"/>
       <c r="P9" s="4" t="inlineStr"/>
-      <c r="Q9" s="9" t="inlineStr"/>
-      <c r="R9" s="9" t="inlineStr"/>
+      <c r="Q9" s="7" t="inlineStr"/>
+      <c r="R9" s="7" t="inlineStr"/>
       <c r="S9" s="4" t="inlineStr"/>
       <c r="T9" s="4" t="inlineStr"/>
       <c r="U9" s="4" t="inlineStr"/>
       <c r="V9" s="4" t="inlineStr"/>
       <c r="W9" s="4" t="inlineStr"/>
-      <c r="X9" s="9" t="inlineStr"/>
-      <c r="Y9" s="9" t="inlineStr"/>
+      <c r="X9" s="7" t="inlineStr"/>
+      <c r="Y9" s="7" t="inlineStr"/>
       <c r="Z9" s="4" t="inlineStr"/>
       <c r="AA9" s="4" t="inlineStr"/>
       <c r="AB9" s="4" t="inlineStr"/>
       <c r="AC9" s="4" t="inlineStr"/>
       <c r="AD9" s="4" t="inlineStr"/>
-      <c r="AE9" s="9" t="inlineStr"/>
-      <c r="AF9" s="9" t="inlineStr"/>
+      <c r="AE9" s="7" t="inlineStr"/>
+      <c r="AF9" s="7" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="8" t="n"/>
       <c r="B10" s="4" t="inlineStr"/>
-      <c r="C10" s="9" t="inlineStr"/>
-      <c r="D10" s="9" t="inlineStr"/>
+      <c r="C10" s="7" t="inlineStr"/>
+      <c r="D10" s="7" t="inlineStr"/>
       <c r="E10" s="4" t="inlineStr"/>
       <c r="F10" s="4" t="inlineStr"/>
       <c r="G10" s="4" t="inlineStr"/>
       <c r="H10" s="4" t="inlineStr"/>
       <c r="I10" s="4" t="inlineStr"/>
-      <c r="J10" s="9" t="inlineStr"/>
-      <c r="K10" s="9" t="inlineStr"/>
+      <c r="J10" s="7" t="inlineStr"/>
+      <c r="K10" s="7" t="inlineStr"/>
       <c r="L10" s="4" t="inlineStr"/>
       <c r="M10" s="4" t="inlineStr"/>
       <c r="N10" s="4" t="inlineStr"/>
       <c r="O10" s="4" t="inlineStr"/>
       <c r="P10" s="4" t="inlineStr"/>
-      <c r="Q10" s="9" t="inlineStr"/>
-      <c r="R10" s="9" t="inlineStr"/>
+      <c r="Q10" s="7" t="inlineStr"/>
+      <c r="R10" s="7" t="inlineStr"/>
       <c r="S10" s="4" t="inlineStr"/>
       <c r="T10" s="4" t="inlineStr"/>
       <c r="U10" s="4" t="inlineStr"/>
       <c r="V10" s="4" t="inlineStr"/>
       <c r="W10" s="4" t="inlineStr"/>
-      <c r="X10" s="9" t="inlineStr"/>
-      <c r="Y10" s="9" t="inlineStr"/>
+      <c r="X10" s="7" t="inlineStr"/>
+      <c r="Y10" s="7" t="inlineStr"/>
       <c r="Z10" s="4" t="inlineStr"/>
       <c r="AA10" s="4" t="inlineStr"/>
       <c r="AB10" s="4" t="inlineStr"/>
       <c r="AC10" s="4" t="inlineStr"/>
       <c r="AD10" s="4" t="inlineStr"/>
-      <c r="AE10" s="9" t="inlineStr"/>
-      <c r="AF10" s="9" t="inlineStr"/>
+      <c r="AE10" s="7" t="inlineStr"/>
+      <c r="AF10" s="7" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="8" t="n"/>
       <c r="B11" s="4" t="inlineStr"/>
-      <c r="C11" s="9" t="inlineStr"/>
-      <c r="D11" s="9" t="inlineStr"/>
+      <c r="C11" s="7" t="inlineStr"/>
+      <c r="D11" s="7" t="inlineStr"/>
       <c r="E11" s="4" t="inlineStr"/>
       <c r="F11" s="4" t="inlineStr"/>
       <c r="G11" s="4" t="inlineStr"/>
       <c r="H11" s="4" t="inlineStr"/>
       <c r="I11" s="4" t="inlineStr"/>
-      <c r="J11" s="9" t="inlineStr"/>
-      <c r="K11" s="9" t="inlineStr"/>
+      <c r="J11" s="7" t="inlineStr"/>
+      <c r="K11" s="7" t="inlineStr"/>
       <c r="L11" s="4" t="inlineStr"/>
       <c r="M11" s="4" t="inlineStr"/>
       <c r="N11" s="4" t="inlineStr"/>
       <c r="O11" s="4" t="inlineStr"/>
       <c r="P11" s="4" t="inlineStr"/>
-      <c r="Q11" s="9" t="inlineStr"/>
-      <c r="R11" s="9" t="inlineStr"/>
+      <c r="Q11" s="7" t="inlineStr"/>
+      <c r="R11" s="7" t="inlineStr"/>
       <c r="S11" s="4" t="inlineStr"/>
       <c r="T11" s="4" t="inlineStr"/>
       <c r="U11" s="4" t="inlineStr"/>
       <c r="V11" s="4" t="inlineStr"/>
       <c r="W11" s="4" t="inlineStr"/>
-      <c r="X11" s="9" t="inlineStr"/>
-      <c r="Y11" s="9" t="inlineStr"/>
+      <c r="X11" s="7" t="inlineStr"/>
+      <c r="Y11" s="7" t="inlineStr"/>
       <c r="Z11" s="4" t="inlineStr"/>
       <c r="AA11" s="4" t="inlineStr"/>
       <c r="AB11" s="4" t="inlineStr"/>
       <c r="AC11" s="4" t="inlineStr"/>
       <c r="AD11" s="4" t="inlineStr"/>
-      <c r="AE11" s="9" t="inlineStr"/>
-      <c r="AF11" s="9" t="inlineStr"/>
+      <c r="AE11" s="7" t="inlineStr"/>
+      <c r="AF11" s="7" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="8" t="n"/>
       <c r="B12" s="4" t="inlineStr"/>
-      <c r="C12" s="9" t="inlineStr"/>
-      <c r="D12" s="9" t="inlineStr"/>
+      <c r="C12" s="7" t="inlineStr"/>
+      <c r="D12" s="7" t="inlineStr"/>
       <c r="E12" s="4" t="inlineStr"/>
       <c r="F12" s="4" t="inlineStr"/>
       <c r="G12" s="4" t="inlineStr"/>
       <c r="H12" s="4" t="inlineStr"/>
       <c r="I12" s="4" t="inlineStr"/>
-      <c r="J12" s="9" t="inlineStr"/>
-      <c r="K12" s="9" t="inlineStr"/>
+      <c r="J12" s="7" t="inlineStr"/>
+      <c r="K12" s="7" t="inlineStr"/>
       <c r="L12" s="4" t="inlineStr"/>
       <c r="M12" s="4" t="inlineStr"/>
       <c r="N12" s="4" t="inlineStr"/>
       <c r="O12" s="4" t="inlineStr"/>
       <c r="P12" s="4" t="inlineStr"/>
-      <c r="Q12" s="9" t="inlineStr"/>
-      <c r="R12" s="9" t="inlineStr"/>
+      <c r="Q12" s="7" t="inlineStr"/>
+      <c r="R12" s="7" t="inlineStr"/>
       <c r="S12" s="4" t="inlineStr"/>
       <c r="T12" s="4" t="inlineStr"/>
       <c r="U12" s="4" t="inlineStr"/>
       <c r="V12" s="4" t="inlineStr"/>
       <c r="W12" s="4" t="inlineStr"/>
-      <c r="X12" s="9" t="inlineStr"/>
-      <c r="Y12" s="9" t="inlineStr"/>
+      <c r="X12" s="7" t="inlineStr"/>
+      <c r="Y12" s="7" t="inlineStr"/>
       <c r="Z12" s="4" t="inlineStr"/>
       <c r="AA12" s="4" t="inlineStr"/>
       <c r="AB12" s="4" t="inlineStr"/>
       <c r="AC12" s="4" t="inlineStr"/>
       <c r="AD12" s="4" t="inlineStr"/>
-      <c r="AE12" s="9" t="inlineStr"/>
-      <c r="AF12" s="9" t="inlineStr"/>
+      <c r="AE12" s="7" t="inlineStr"/>
+      <c r="AF12" s="7" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="8" t="n"/>
       <c r="B13" s="4" t="inlineStr"/>
-      <c r="C13" s="9" t="inlineStr"/>
-      <c r="D13" s="9" t="inlineStr"/>
+      <c r="C13" s="7" t="inlineStr"/>
+      <c r="D13" s="7" t="inlineStr"/>
       <c r="E13" s="4" t="inlineStr"/>
       <c r="F13" s="4" t="inlineStr"/>
       <c r="G13" s="4" t="inlineStr"/>
       <c r="H13" s="4" t="inlineStr"/>
       <c r="I13" s="4" t="inlineStr"/>
-      <c r="J13" s="9" t="inlineStr"/>
-      <c r="K13" s="9" t="inlineStr"/>
+      <c r="J13" s="7" t="inlineStr"/>
+      <c r="K13" s="7" t="inlineStr"/>
       <c r="L13" s="4" t="inlineStr"/>
       <c r="M13" s="4" t="inlineStr"/>
       <c r="N13" s="4" t="inlineStr"/>
       <c r="O13" s="4" t="inlineStr"/>
       <c r="P13" s="4" t="inlineStr"/>
-      <c r="Q13" s="9" t="inlineStr"/>
-      <c r="R13" s="9" t="inlineStr"/>
+      <c r="Q13" s="7" t="inlineStr"/>
+      <c r="R13" s="7" t="inlineStr"/>
       <c r="S13" s="4" t="inlineStr"/>
       <c r="T13" s="4" t="inlineStr"/>
       <c r="U13" s="4" t="inlineStr"/>
       <c r="V13" s="4" t="inlineStr"/>
       <c r="W13" s="4" t="inlineStr"/>
-      <c r="X13" s="9" t="inlineStr"/>
-      <c r="Y13" s="9" t="inlineStr"/>
+      <c r="X13" s="7" t="inlineStr"/>
+      <c r="Y13" s="7" t="inlineStr"/>
       <c r="Z13" s="4" t="inlineStr"/>
       <c r="AA13" s="4" t="inlineStr"/>
       <c r="AB13" s="4" t="inlineStr"/>
       <c r="AC13" s="4" t="inlineStr"/>
       <c r="AD13" s="4" t="inlineStr"/>
-      <c r="AE13" s="9" t="inlineStr"/>
-      <c r="AF13" s="9" t="inlineStr"/>
+      <c r="AE13" s="7" t="inlineStr"/>
+      <c r="AF13" s="7" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="8" t="n"/>
       <c r="B14" s="4" t="inlineStr"/>
-      <c r="C14" s="9" t="inlineStr"/>
-      <c r="D14" s="9" t="inlineStr"/>
+      <c r="C14" s="7" t="inlineStr"/>
+      <c r="D14" s="7" t="inlineStr"/>
       <c r="E14" s="4" t="inlineStr"/>
       <c r="F14" s="4" t="inlineStr"/>
       <c r="G14" s="4" t="inlineStr"/>
       <c r="H14" s="4" t="inlineStr"/>
       <c r="I14" s="4" t="inlineStr"/>
-      <c r="J14" s="9" t="inlineStr"/>
-      <c r="K14" s="9" t="inlineStr"/>
+      <c r="J14" s="7" t="inlineStr"/>
+      <c r="K14" s="7" t="inlineStr"/>
       <c r="L14" s="4" t="inlineStr"/>
       <c r="M14" s="4" t="inlineStr"/>
       <c r="N14" s="4" t="inlineStr"/>
       <c r="O14" s="4" t="inlineStr"/>
       <c r="P14" s="4" t="inlineStr"/>
-      <c r="Q14" s="9" t="inlineStr"/>
-      <c r="R14" s="9" t="inlineStr"/>
+      <c r="Q14" s="7" t="inlineStr"/>
+      <c r="R14" s="7" t="inlineStr"/>
       <c r="S14" s="4" t="inlineStr"/>
       <c r="T14" s="4" t="inlineStr"/>
       <c r="U14" s="4" t="inlineStr"/>
       <c r="V14" s="4" t="inlineStr"/>
       <c r="W14" s="4" t="inlineStr"/>
-      <c r="X14" s="9" t="inlineStr"/>
-      <c r="Y14" s="9" t="inlineStr"/>
+      <c r="X14" s="7" t="inlineStr"/>
+      <c r="Y14" s="7" t="inlineStr"/>
       <c r="Z14" s="4" t="inlineStr"/>
       <c r="AA14" s="4" t="inlineStr"/>
       <c r="AB14" s="4" t="inlineStr"/>
       <c r="AC14" s="4" t="inlineStr"/>
       <c r="AD14" s="4" t="inlineStr"/>
-      <c r="AE14" s="9" t="inlineStr"/>
-      <c r="AF14" s="9" t="inlineStr"/>
+      <c r="AE14" s="7" t="inlineStr"/>
+      <c r="AF14" s="7" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="8" t="n"/>
       <c r="B15" s="4" t="inlineStr"/>
-      <c r="C15" s="9" t="inlineStr"/>
-      <c r="D15" s="9" t="inlineStr"/>
+      <c r="C15" s="7" t="inlineStr"/>
+      <c r="D15" s="7" t="inlineStr"/>
       <c r="E15" s="4" t="inlineStr"/>
       <c r="F15" s="4" t="inlineStr"/>
       <c r="G15" s="4" t="inlineStr"/>
       <c r="H15" s="4" t="inlineStr"/>
       <c r="I15" s="4" t="inlineStr"/>
-      <c r="J15" s="9" t="inlineStr"/>
-      <c r="K15" s="9" t="inlineStr"/>
+      <c r="J15" s="7" t="inlineStr"/>
+      <c r="K15" s="7" t="inlineStr"/>
       <c r="L15" s="4" t="inlineStr"/>
       <c r="M15" s="4" t="inlineStr"/>
       <c r="N15" s="4" t="inlineStr"/>
       <c r="O15" s="4" t="inlineStr"/>
       <c r="P15" s="4" t="inlineStr"/>
-      <c r="Q15" s="9" t="inlineStr"/>
-      <c r="R15" s="9" t="inlineStr"/>
+      <c r="Q15" s="7" t="inlineStr"/>
+      <c r="R15" s="7" t="inlineStr"/>
       <c r="S15" s="4" t="inlineStr"/>
       <c r="T15" s="4" t="inlineStr"/>
       <c r="U15" s="4" t="inlineStr"/>
       <c r="V15" s="4" t="inlineStr"/>
       <c r="W15" s="4" t="inlineStr"/>
-      <c r="X15" s="9" t="inlineStr"/>
-      <c r="Y15" s="9" t="inlineStr"/>
+      <c r="X15" s="7" t="inlineStr"/>
+      <c r="Y15" s="7" t="inlineStr"/>
       <c r="Z15" s="4" t="inlineStr"/>
       <c r="AA15" s="4" t="inlineStr"/>
       <c r="AB15" s="4" t="inlineStr"/>
       <c r="AC15" s="4" t="inlineStr"/>
       <c r="AD15" s="4" t="inlineStr"/>
-      <c r="AE15" s="9" t="inlineStr"/>
-      <c r="AF15" s="9" t="inlineStr"/>
+      <c r="AE15" s="7" t="inlineStr"/>
+      <c r="AF15" s="7" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="8" t="n"/>
       <c r="B16" s="4" t="inlineStr"/>
-      <c r="C16" s="9" t="inlineStr"/>
-      <c r="D16" s="9" t="inlineStr"/>
+      <c r="C16" s="7" t="inlineStr"/>
+      <c r="D16" s="7" t="inlineStr"/>
       <c r="E16" s="4" t="inlineStr"/>
       <c r="F16" s="4" t="inlineStr"/>
       <c r="G16" s="4" t="inlineStr"/>
       <c r="H16" s="4" t="inlineStr"/>
       <c r="I16" s="4" t="inlineStr"/>
-      <c r="J16" s="9" t="inlineStr"/>
-      <c r="K16" s="9" t="inlineStr"/>
+      <c r="J16" s="7" t="inlineStr"/>
+      <c r="K16" s="7" t="inlineStr"/>
       <c r="L16" s="4" t="inlineStr"/>
       <c r="M16" s="4" t="inlineStr"/>
       <c r="N16" s="4" t="inlineStr"/>
       <c r="O16" s="4" t="inlineStr"/>
       <c r="P16" s="4" t="inlineStr"/>
-      <c r="Q16" s="9" t="inlineStr"/>
-      <c r="R16" s="9" t="inlineStr"/>
+      <c r="Q16" s="7" t="inlineStr"/>
+      <c r="R16" s="7" t="inlineStr"/>
       <c r="S16" s="4" t="inlineStr"/>
       <c r="T16" s="4" t="inlineStr"/>
       <c r="U16" s="4" t="inlineStr"/>
       <c r="V16" s="4" t="inlineStr"/>
       <c r="W16" s="4" t="inlineStr"/>
-      <c r="X16" s="9" t="inlineStr"/>
-      <c r="Y16" s="9" t="inlineStr"/>
+      <c r="X16" s="7" t="inlineStr"/>
+      <c r="Y16" s="7" t="inlineStr"/>
       <c r="Z16" s="4" t="inlineStr"/>
       <c r="AA16" s="4" t="inlineStr"/>
       <c r="AB16" s="4" t="inlineStr"/>
       <c r="AC16" s="4" t="inlineStr"/>
       <c r="AD16" s="4" t="inlineStr"/>
-      <c r="AE16" s="9" t="inlineStr"/>
-      <c r="AF16" s="9" t="inlineStr"/>
+      <c r="AE16" s="7" t="inlineStr"/>
+      <c r="AF16" s="7" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="8" t="n"/>
       <c r="B17" s="4" t="inlineStr"/>
-      <c r="C17" s="9" t="inlineStr"/>
-      <c r="D17" s="9" t="inlineStr"/>
+      <c r="C17" s="7" t="inlineStr"/>
+      <c r="D17" s="7" t="inlineStr"/>
       <c r="E17" s="4" t="inlineStr"/>
       <c r="F17" s="4" t="inlineStr"/>
       <c r="G17" s="4" t="inlineStr"/>
       <c r="H17" s="4" t="inlineStr"/>
       <c r="I17" s="4" t="inlineStr"/>
-      <c r="J17" s="9" t="inlineStr"/>
-      <c r="K17" s="9" t="inlineStr"/>
+      <c r="J17" s="7" t="inlineStr"/>
+      <c r="K17" s="7" t="inlineStr"/>
       <c r="L17" s="4" t="inlineStr"/>
       <c r="M17" s="4" t="inlineStr"/>
       <c r="N17" s="4" t="inlineStr"/>
       <c r="O17" s="4" t="inlineStr"/>
       <c r="P17" s="4" t="inlineStr"/>
-      <c r="Q17" s="9" t="inlineStr"/>
-      <c r="R17" s="9" t="inlineStr"/>
+      <c r="Q17" s="7" t="inlineStr"/>
+      <c r="R17" s="7" t="inlineStr"/>
       <c r="S17" s="4" t="inlineStr"/>
       <c r="T17" s="4" t="inlineStr"/>
       <c r="U17" s="4" t="inlineStr"/>
       <c r="V17" s="4" t="inlineStr"/>
       <c r="W17" s="4" t="inlineStr"/>
-      <c r="X17" s="9" t="inlineStr"/>
-      <c r="Y17" s="9" t="inlineStr"/>
+      <c r="X17" s="7" t="inlineStr"/>
+      <c r="Y17" s="7" t="inlineStr"/>
       <c r="Z17" s="4" t="inlineStr"/>
       <c r="AA17" s="4" t="inlineStr"/>
       <c r="AB17" s="4" t="inlineStr"/>
       <c r="AC17" s="4" t="inlineStr"/>
       <c r="AD17" s="4" t="inlineStr"/>
-      <c r="AE17" s="9" t="inlineStr"/>
-      <c r="AF17" s="9" t="inlineStr"/>
+      <c r="AE17" s="7" t="inlineStr"/>
+      <c r="AF17" s="7" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="8" t="n"/>
       <c r="B18" s="4" t="inlineStr"/>
-      <c r="C18" s="9" t="inlineStr"/>
-      <c r="D18" s="9" t="inlineStr"/>
+      <c r="C18" s="7" t="inlineStr"/>
+      <c r="D18" s="7" t="inlineStr"/>
       <c r="E18" s="4" t="inlineStr"/>
       <c r="F18" s="4" t="inlineStr"/>
       <c r="G18" s="4" t="inlineStr"/>
       <c r="H18" s="4" t="inlineStr"/>
       <c r="I18" s="4" t="inlineStr"/>
-      <c r="J18" s="9" t="inlineStr"/>
-      <c r="K18" s="9" t="inlineStr"/>
+      <c r="J18" s="7" t="inlineStr"/>
+      <c r="K18" s="7" t="inlineStr"/>
       <c r="L18" s="4" t="inlineStr"/>
       <c r="M18" s="4" t="inlineStr"/>
       <c r="N18" s="4" t="inlineStr"/>
       <c r="O18" s="4" t="inlineStr"/>
       <c r="P18" s="4" t="inlineStr"/>
-      <c r="Q18" s="9" t="inlineStr"/>
-      <c r="R18" s="9" t="inlineStr"/>
+      <c r="Q18" s="7" t="inlineStr"/>
+      <c r="R18" s="7" t="inlineStr"/>
       <c r="S18" s="4" t="inlineStr"/>
       <c r="T18" s="4" t="inlineStr"/>
       <c r="U18" s="4" t="inlineStr"/>
       <c r="V18" s="4" t="inlineStr"/>
       <c r="W18" s="4" t="inlineStr"/>
-      <c r="X18" s="9" t="inlineStr"/>
-      <c r="Y18" s="9" t="inlineStr"/>
+      <c r="X18" s="7" t="inlineStr"/>
+      <c r="Y18" s="7" t="inlineStr"/>
       <c r="Z18" s="4" t="inlineStr"/>
       <c r="AA18" s="4" t="inlineStr"/>
       <c r="AB18" s="4" t="inlineStr"/>
       <c r="AC18" s="4" t="inlineStr"/>
       <c r="AD18" s="4" t="inlineStr"/>
-      <c r="AE18" s="9" t="inlineStr"/>
-      <c r="AF18" s="9" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="8" t="n"/>
-      <c r="B19" s="4" t="inlineStr"/>
-      <c r="C19" s="9" t="inlineStr"/>
-      <c r="D19" s="9" t="inlineStr"/>
-      <c r="E19" s="4" t="inlineStr"/>
-      <c r="F19" s="4" t="inlineStr"/>
-      <c r="G19" s="4" t="inlineStr"/>
-      <c r="H19" s="4" t="inlineStr"/>
-      <c r="I19" s="4" t="inlineStr"/>
-      <c r="J19" s="9" t="inlineStr"/>
-      <c r="K19" s="9" t="inlineStr"/>
-      <c r="L19" s="4" t="inlineStr"/>
-      <c r="M19" s="4" t="inlineStr"/>
-      <c r="N19" s="4" t="inlineStr"/>
-      <c r="O19" s="4" t="inlineStr"/>
-      <c r="P19" s="4" t="inlineStr"/>
-      <c r="Q19" s="9" t="inlineStr"/>
-      <c r="R19" s="9" t="inlineStr"/>
-      <c r="S19" s="4" t="inlineStr"/>
-      <c r="T19" s="4" t="inlineStr"/>
-      <c r="U19" s="4" t="inlineStr"/>
-      <c r="V19" s="4" t="inlineStr"/>
-      <c r="W19" s="4" t="inlineStr"/>
-      <c r="X19" s="9" t="inlineStr"/>
-      <c r="Y19" s="9" t="inlineStr"/>
-      <c r="Z19" s="4" t="inlineStr"/>
-      <c r="AA19" s="4" t="inlineStr"/>
-      <c r="AB19" s="4" t="inlineStr"/>
-      <c r="AC19" s="4" t="inlineStr"/>
-      <c r="AD19" s="4" t="inlineStr"/>
-      <c r="AE19" s="9" t="inlineStr"/>
-      <c r="AF19" s="9" t="inlineStr"/>
+      <c r="AE18" s="7" t="inlineStr"/>
+      <c r="AF18" s="7" t="inlineStr"/>
     </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="2">
     <mergeCell ref="A2"/>
-    <mergeCell ref="B3:AF3"/>
     <mergeCell ref="A1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>